<commit_message>
File change | clean
</commit_message>
<xml_diff>
--- a/data/flo/fabric-invoice-numbers.xlsx
+++ b/data/flo/fabric-invoice-numbers.xlsx
@@ -66,12 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -382,7 +385,7 @@
   <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="14.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -392,12 +395,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="2">
-        <v>1010050400</v>
+        <v>1010050763</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="2">
-        <v>1010050399</v>
+      <c r="A3" s="3">
+        <v>1010050764</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">

</xml_diff>